<commit_message>
Updated results for reproductioin.
</commit_message>
<xml_diff>
--- a/results/02_taxa_assemblage/artifacts/02_hindsight_updated_data.xlsx
+++ b/results/02_taxa_assemblage/artifacts/02_hindsight_updated_data.xlsx
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="B173" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174">
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="B193" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="B195" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196">
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="B199" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="200">
@@ -2108,7 +2108,7 @@
         </is>
       </c>
       <c r="B200" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -2214,7 +2214,7 @@
         </is>
       </c>
       <c r="B212" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="213">

</xml_diff>